<commit_message>
Add 5 deterministic edge cases + native PDF extraction
- PDF-direct extraction: whole PDF as single document content block to Opus 4.7
- Edge 1: partial/split invoicing with cumulative PO balance
- Edge 2: vendor identity mismatch (authoritative id first, fuzzy name fallback)
- Edge 3: inconsistent item naming (deterministic alias map)
- Edge 4: true duplicate detection (vendor + invoice# + PO + amount within 0.1%)
- Edge 5: credit note branch (never auto-approves, links to referenced invoice)
- Plus amount-over-tolerance and no-PO demo invoices
- 9 new sample PDFs + 4 new PO rows in po_master

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-invoices/po_master.xlsx
+++ b/sample-invoices/po_master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1153,6 +1153,146 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PO-2001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Bharat Auto Spares</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GST-27AABCB1234M1Z5</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Consulting engagement - Milestone 1; Consulting engagement - Milestone 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PO-2002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Kumar Traders</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PAN-AAAPK1234C</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Q3 consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PO-2003</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Volkswagen Components India</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GST-06AAACV5566H1ZP</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>New Kushaq</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PO-2004</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Local Cartons Co</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GST-27AABLC2233N1ZY</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Carton stock replenishment</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>